<commit_message>
fix: reminder email states real minutes left; update black-box table
- Late-approved bookings get the reminder right away, but the subject and
  heading always said 'อีก 15 นาที'; use the actual minutes left
- Test_Cases_BlockTest_Result.xlsx still listed T23-T25 as check-in cases,
  a feature removed in 7633d63; replace with the current cancel / early
  release cases from tests_blocktest.py and refresh the summary sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test_Cases_BlockTest_Result.xlsx
+++ b/Test_Cases_BlockTest_Result.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="สรุปผล" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปผล" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$G$31</definedName>
@@ -1310,22 +1310,22 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>เช็คอิน</t>
+          <t>ยกเลิกการจอง</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>การจองที่อนุมัติแล้ว กดเช็คอิน 15 นาทีก่อนเวลาเริ่ม</t>
+          <t>การจองที่อนุมัติแล้ว ยกเลิกก่อนถึงเวลาเริ่ม 10 นาที</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>สำเร็จ สถานะเปลี่ยนเป็น "เช็คอินแล้ว"</t>
+          <t>ยกเลิกสำเร็จ สถานะเปลี่ยนเป็น "ยกเลิกแล้ว"</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200 {"message": "Check-in สำเร็จ", "status": "checked_in"} สถานะเปลี่ยนเป็น checked_in</t>
+          <t>HTTP 200 {"message": "ยกเลิกการจองเรียบร้อยแล้ว", "result": "cancelled"} สถานะเปลี่ยนเป็น cancelled</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1333,11 +1333,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>ขอบเขตหน้าต่างเช็คอินคือ 15 นาทีก่อนเวลาเริ่ม ทดสอบคู่กับ T24</t>
-        </is>
-      </c>
+      <c r="G24" s="3" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1347,22 +1343,22 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>เช็คอิน</t>
+          <t>คืนห้องก่อนเวลา</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>การจองที่อนุมัติแล้ว กดเช็คอิน 16 นาทีก่อนเวลาเริ่ม</t>
+          <t>การจองที่กำลังใช้งานอยู่ (เริ่มไปแล้ว 30 นาที) กดยกเลิก</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>ปฏิเสธ ยังไม่ถึงเวลาเช็คอิน</t>
+          <t>คืนห้องก่อนเวลา สถานะยังเป็นอนุมัติ เวลาสิ้นสุดเลื่อนเป็นเวลาปัจจุบัน และช่วงที่เหลือผู้อื่นจองต่อได้</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400 {"error": "ยังไม่ถึงเวลา Check-in", "check_in_available_at": "..."} สถานะยังเป็น approved</t>
+          <t>HTTP 200 {"message": "คืนห้องเรียบร้อยแล้ว (สิ้นสุด 21:22 น.)", "result": "released"} สถานะยังเป็น approved เวลาจบเลื่อนเป็นเวลาที่กด และผู้ใช้อื่นจองช่วงที่เหลือได้ (HTTP 201)</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1370,7 +1366,11 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>ระบบไม่มีการเช็คอิน ใช้การคืนห้องก่อนเวลาแทน</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1380,22 +1380,22 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>เช็คอิน</t>
+          <t>ยกเลิกการจอง</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>กดเช็คอินการจองที่ยังรออนุมัติ</t>
+          <t>ยกเลิกการจองที่เวลาสิ้นสุดไปแล้ว</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>ปฏิเสธ และแจ้งสถานะปัจจุบัน</t>
+          <t>ปฏิเสธ "เวลาที่จองสิ้นสุดไปแล้ว"</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400 {"error": "ไม่สามารถ Check-in ได้", "status": "pending"} แจ้งสถานะปัจจุบันกลับมาด้วย</t>
+          <t>HTTP 400 {"error": "ยกเลิกไม่ได้ เวลาที่จองสิ้นสุดไปแล้ว"} สถานะยังเป็น approved</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1403,7 +1403,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="n"/>
     </row>
     <row r="27" ht="46" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>qa_test_bot (นักศึกษา), qa_admin (ผู้ดูแลระบบ), qa_user_b (นักศึกษาอีกคน)</t>
+          <t>qa_test_bot (อาจารย์), qa_admin (ผู้ดูแลระบบ), qa_user_b (นักศึกษา)</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>20 กันยายน 2569</t>
+          <t>16 ตุลาคม 2569</t>
         </is>
       </c>
     </row>

</xml_diff>